<commit_message>
Implement 2026/27 artwork and portable release 2.0.0
</commit_message>
<xml_diff>
--- a/input/ejemplo.xlsx
+++ b/input/ejemplo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Baloncesto\generador_horarios\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmabascal\Downloads\Carlos\Basket Aranjuez\Autobuses y Horarios\2026-2027\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDC9CE1-0C3C-4721-AA0A-CA9956D8734C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{79C8D132-4DA6-49DF-A48B-32E5F1E187AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A18B7C17-1169-4FC5-9717-33F65EDFB014}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10240" xr2:uid="{C1453126-735E-49F0-8EE0-149DC1E154EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
   <si>
     <t>Categoría</t>
   </si>
@@ -40,244 +40,94 @@
     <t>Campo de juego</t>
   </si>
   <si>
+    <t>Alv Fem 1ºaño LIGA MARCO ALDANY</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ RUBIOCAR</t>
+  </si>
+  <si>
+    <t>C.D.I. ROZASBASKET</t>
+  </si>
+  <si>
+    <t>LAS OLIVAS, CIUDAD DEPORTIVA</t>
+  </si>
+  <si>
+    <t>Alv Mas 2ºaño LIGA MARCO ALDANY - PLATA</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ CAS</t>
+  </si>
+  <si>
+    <t>FUENTELARREYNA</t>
+  </si>
+  <si>
+    <t>Alv Fem 2ºaño LIGA MARCO ALDANY - ORO</t>
+  </si>
+  <si>
+    <t>FEMENINO ALCORCON AMARILLO</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ BLANCO</t>
+  </si>
+  <si>
+    <t>LA CANALEJA, PABELLON PISTA 2</t>
+  </si>
+  <si>
+    <t>Junior Masc. Pref.</t>
+  </si>
+  <si>
+    <t>SAN AGUSTIN MADRID "A"</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ MISTER PIXEL</t>
+  </si>
+  <si>
+    <t>SAN AGUSTIN, PABELLON PRINCIPAL</t>
+  </si>
+  <si>
+    <t>Alv Mas 1ºaño LIGA MARCO ALDANY</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ</t>
+  </si>
+  <si>
+    <t>BALONCESTO ARISTOS A</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ C</t>
+  </si>
+  <si>
+    <t>MEJORADA 2012 C.B.</t>
+  </si>
+  <si>
+    <t>Alv Fem 2ºaño LIGA MARCO ALDANY - PLATA</t>
+  </si>
+  <si>
+    <t>BRAINS MORALEJA</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ NEGRO</t>
+  </si>
+  <si>
+    <t>BRAINS LA MORALEJA, COLEGIO</t>
+  </si>
+  <si>
+    <t>BASKET ARANJUEZ D</t>
+  </si>
+  <si>
+    <t>IPANEMA MADRID ELITE BASKETBALL</t>
+  </si>
+  <si>
     <t>Cadete Fem. 1ºaño</t>
   </si>
   <si>
-    <t>BASKET ARANJUEZ BLANCO</t>
-  </si>
-  <si>
-    <t>SAN AGUSTIN MADRID</t>
-  </si>
-  <si>
-    <t>LAS OLIVAS, CIUDAD DEPORTIVA</t>
-  </si>
-  <si>
-    <t>Infantil Fem. 1ºaño</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ AMARILLO</t>
-  </si>
-  <si>
-    <t>ESTUDIO AZUL</t>
-  </si>
-  <si>
-    <t>Cadete Masc. Pref.</t>
-  </si>
-  <si>
-    <t>SANTA MARIA DEL PILAR "A"</t>
-  </si>
-  <si>
-    <t>SANTA MARIA DEL PILAR, PISTA AZUL SEMICUBIERTA</t>
-  </si>
-  <si>
-    <t>ADC BOADILLA "C"</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ NEGRO</t>
-  </si>
-  <si>
-    <t>ANGEL NIETO, COMPLEJO DPTIVO. MPAL.</t>
-  </si>
-  <si>
-    <t>Alv Mas 2ºaño LIGA MARCO ALDANY - ORO</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ CLINICA RICHER</t>
-  </si>
-  <si>
-    <t>REAL CANOE N.C.</t>
-  </si>
-  <si>
-    <t>Infantil Masc. 1ºaño</t>
-  </si>
-  <si>
-    <t>ESTUDIO BLANCO</t>
-  </si>
-  <si>
-    <t>Cadete Fem. Pref.</t>
-  </si>
-  <si>
-    <t>BUEN CONSEJO 10 BLANCO</t>
-  </si>
-  <si>
-    <t>BUEN CONSEJO, PABELLON COLEGIO</t>
-  </si>
-  <si>
-    <t>HYUNDAI ALMOAUTO SAN FERNANDO</t>
-  </si>
-  <si>
-    <t>AGUSTIN MARAÑON, PABELLON</t>
-  </si>
-  <si>
-    <t>Alv Fem 2ºaño LIGA MARCO ALDANY - ORO</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ POSTAS TAPERIA</t>
-  </si>
-  <si>
-    <t>LEGAMAR LEGANÉS</t>
-  </si>
-  <si>
-    <t>Infantil Fem. Pref.</t>
-  </si>
-  <si>
-    <t>BALONCESTO RIVAS SURESTE B</t>
-  </si>
-  <si>
-    <t>CERRO DEL TELEGRAFO, PABELLON</t>
-  </si>
-  <si>
-    <t>Junior Fem. Pref.</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ ESENCIAL SALUD</t>
-  </si>
-  <si>
-    <t>FUNDAL ALCOBENDAS "C"</t>
-  </si>
-  <si>
-    <t>Alv Fem 1ºaño LIGA MARCO ALDANY</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ RUBIOCAR</t>
-  </si>
-  <si>
-    <t>FEMENINO ALCORCON AZUL</t>
-  </si>
-  <si>
-    <t>MAJADAHONDA</t>
-  </si>
-  <si>
-    <t>Alv Fem 2ºaño LIGA MARCO ALDANY - PLATA</t>
-  </si>
-  <si>
-    <t>Infantil Masc. Pref.</t>
-  </si>
-  <si>
-    <t>BALONCESTO ALCALA</t>
-  </si>
-  <si>
-    <t>SAN JOSE DE CALASANZ, COLEGIO</t>
-  </si>
-  <si>
-    <t>Alv Mas 1ºaño LIGA MARCO ALDANY</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ CAS</t>
-  </si>
-  <si>
-    <t>CORAZONISTAS</t>
-  </si>
-  <si>
-    <t>Cadete Masc. 1ºaño</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ</t>
-  </si>
-  <si>
-    <t>Junior Masc. Pref.</t>
-  </si>
-  <si>
-    <t>VILLALBA AMORAGA CATERING</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ A</t>
-  </si>
-  <si>
-    <t>LOS NEGRALES, POLIDEPORTIVO</t>
-  </si>
-  <si>
-    <t>PARQUE CATALUÑA TORREJÓN AMARILLO</t>
-  </si>
-  <si>
-    <t>COLEGIO ALAMEDA DE OSUNA "A"</t>
-  </si>
-  <si>
-    <t>VALCUDE ALCOBENDAS</t>
-  </si>
-  <si>
-    <t>ARROYOMOLINOS C.B. "A"</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ B</t>
-  </si>
-  <si>
-    <t>LOS MOSQUITOS, PABELLON</t>
-  </si>
-  <si>
-    <t>2ª Div Aut Masc ORO</t>
-  </si>
-  <si>
-    <t>MENESIANO</t>
-  </si>
-  <si>
-    <t>BASKET ARANJUEZ A MISTER PIXEL</t>
-  </si>
-  <si>
-    <t>MENESIANO, PABELLON COLEGIO</t>
-  </si>
-  <si>
-    <t>Sub 22 Masc. BRONCE</t>
-  </si>
-  <si>
-    <t>HUMANES CLUB BASKET</t>
-  </si>
-  <si>
-    <t>CAMPOHERMOSO, PABELLON</t>
-  </si>
-  <si>
-    <t>SAN JOSE DEL PARQUE</t>
-  </si>
-  <si>
-    <t>SAN JOSE DEL PARQUE, PABELLON COLEGIO</t>
-  </si>
-  <si>
-    <t>2ª Div Aut Fem PLATA</t>
-  </si>
-  <si>
-    <t>C.B. PERALES</t>
-  </si>
-  <si>
-    <t>Infantil Masculino LIGA AHORRAMAS - PLATA/BRONCE</t>
-  </si>
-  <si>
-    <t>C.D.I. ROZASBASKET BOOSTERS</t>
-  </si>
-  <si>
-    <t>I.E.S. JOSE GARCIA NIETO, PABELLON</t>
-  </si>
-  <si>
-    <t>2ª Div Aut Fem ORO</t>
-  </si>
-  <si>
-    <t>LIONS BASKET ARROYOMOLINOS</t>
-  </si>
-  <si>
-    <t>ANGEL DURANGO, PDVO. MPAL.</t>
-  </si>
-  <si>
-    <t>2ª Div Aut Masc PLATA</t>
-  </si>
-  <si>
-    <t>MADRID ELITE BASKETBALL BLANCO</t>
-  </si>
-  <si>
-    <t>ESTUDIANTES LAS TABLAS, COLEGIO</t>
-  </si>
-  <si>
-    <t>C.B. CIUDAD DE MÓSTOLES</t>
-  </si>
-  <si>
-    <t>LOS ROSALES, PABELLON</t>
-  </si>
-  <si>
-    <t>LOYOLA ARANJUEZ MUELACAR</t>
-  </si>
-  <si>
-    <t>ARROYOMOLINOS C.B.</t>
-  </si>
-  <si>
-    <t>FEMENINO FUENLABRADA</t>
+    <t>BASKET ARANJUEZ D12 SPORT CLINIC</t>
+  </si>
+  <si>
+    <t>BOADILLA MONSTERS</t>
+  </si>
+  <si>
+    <t>Liga Ginos Femenina</t>
   </si>
 </sst>
 </file>
@@ -435,7 +285,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -613,12 +463,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -782,7 +626,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -797,15 +641,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -854,6 +689,44 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="8">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -970,44 +843,6 @@
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1022,15 +857,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C0741B35-1E05-46A6-BC59-B9F1C1BA1347}" name="Tabla1" displayName="Tabla1" ref="A1:F33" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="A1:F33" xr:uid="{C0741B35-1E05-46A6-BC59-B9F1C1BA1347}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{476DE131-5D2A-4B12-890F-8E60EEB92D50}" name="Tabla1" displayName="Tabla1" ref="A1:F11" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:F11" xr:uid="{476DE131-5D2A-4B12-890F-8E60EEB92D50}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{75D3C7B5-DD25-48AE-B247-BCB38F350326}" name="Categoría" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{8A3D3763-1082-4F98-AA54-B4509166E4C4}" name="Local" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{008D13F2-F1BF-4565-9D8E-FC3DBC269721}" name="Visitante" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{02871EA2-EF00-40BB-B2A7-B19E1A5C5BCF}" name="Fecha" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C7D2BBAF-8D58-430C-B373-AE6F42FBAA62}" name="Hora" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{CB059037-A039-4E1B-A4CA-F97D30AA95FE}" name="Campo de juego" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{405B749F-E570-4AF5-BD64-688F1DB332F1}" name="Categoría" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00394F6B-1A8A-418A-95F8-AF8F667D233E}" name="Local" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{DEDE2185-7F98-46AE-8A48-E4CAD7FF0903}" name="Visitante" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{8FAEAA51-64AB-4061-B893-3A47C95BB0CD}" name="Fecha" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{1E60853E-D0CD-4A6C-8F0B-35804BC3C0D9}" name="Hora" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{084553AA-5F87-461A-99F6-1E39B60CBA0A}" name="Campo de juego" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1352,19 +1187,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5ED0CB4-0F3D-4EB5-A706-B7377F5E4F94}">
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB1B1236-8039-4DD0-AEB6-6069D19E9191}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="34.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.44140625" customWidth="1"/>
-    <col min="6" max="6" width="34.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.453125" customWidth="1"/>
+    <col min="6" max="6" width="28.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1385,7 +1220,7 @@
       </c>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1396,7 +1231,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4">
-        <v>46123</v>
+        <v>46305</v>
       </c>
       <c r="E2" s="5">
         <v>0.375</v>
@@ -1406,7 +1241,7 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="26.5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
@@ -1417,7 +1252,7 @@
         <v>12</v>
       </c>
       <c r="D3" s="4">
-        <v>46123</v>
+        <v>46305</v>
       </c>
       <c r="E3" s="5">
         <v>0.375</v>
@@ -1427,7 +1262,7 @@
       </c>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
@@ -1435,627 +1270,165 @@
         <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D4" s="4">
-        <v>46123</v>
+        <v>46305</v>
       </c>
       <c r="E4" s="5">
-        <v>0.44791666666666669</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="26.5" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D5" s="4">
-        <v>46123</v>
+        <v>46305</v>
       </c>
       <c r="E5" s="5">
         <v>0.44791666666666669</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="6" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="7">
-        <v>46123</v>
-      </c>
-      <c r="E6" s="8">
+      <c r="B6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="4">
+        <v>46305</v>
+      </c>
+      <c r="E6" s="5">
         <v>0.45833333333333331</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="7">
-        <v>46123</v>
-      </c>
-      <c r="E7" s="8">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="4">
+        <v>46305</v>
+      </c>
+      <c r="E7" s="5">
         <v>0.45833333333333331</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="26.5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="D8" s="4">
-        <v>46123</v>
+        <v>46305</v>
       </c>
       <c r="E8" s="5">
         <v>0.46875</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="26.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D9" s="4">
-        <v>46123</v>
+        <v>46305</v>
       </c>
       <c r="E9" s="5">
-        <v>0.52083333333333337</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="7">
-        <v>46123</v>
-      </c>
-      <c r="E10" s="8">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="F10" s="6" t="s">
+    <row r="10" spans="1:7" ht="26.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46305</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="26.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D11" s="4">
-        <v>46123</v>
+        <v>46306</v>
       </c>
       <c r="E11" s="5">
-        <v>0.54166666666666663</v>
+        <v>0.44791666666666669</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="7">
-        <v>46123</v>
-      </c>
-      <c r="E12" s="8">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E13" s="5">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="7">
-        <v>46123</v>
-      </c>
-      <c r="E14" s="8">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E15" s="5">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E16" s="5">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E17" s="5">
-        <v>0.75</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E18" s="5">
-        <v>0.75</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="7">
-        <v>46123</v>
-      </c>
-      <c r="E19" s="8">
-        <v>0.75</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D20" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E20" s="5">
-        <v>0.82291666666666663</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" s="7">
-        <v>46123</v>
-      </c>
-      <c r="E21" s="8">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D22" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E22" s="5">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" s="4">
-        <v>46123</v>
-      </c>
-      <c r="E23" s="5">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D24" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E24" s="5">
-        <v>0.46875</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D25" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E25" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E26" s="5">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D27" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E27" s="5">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G27" s="2"/>
-    </row>
-    <row r="28" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E28" s="5">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D29" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E29" s="5">
-        <v>0.55208333333333337</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="G29" s="2"/>
-    </row>
-    <row r="30" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D30" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E30" s="5">
-        <v>0.55208333333333337</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G30" s="2"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D31" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E31" s="5">
-        <v>0.625</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="G31" s="2"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D32" s="4">
-        <v>46124</v>
-      </c>
-      <c r="E32" s="5">
-        <v>0.70833333333333337</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G32" s="2"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="D33" s="7">
-        <v>46124</v>
-      </c>
-      <c r="E33" s="8">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G33" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>